<commit_message>
feat: process_price_mismatches() เพิ่ม logic
เพิ่ม logic ในการ ปรับ oc dc ตามค่า oc/dc amount ตามในไฟล์ cp_data.xlsx เพิ่มด้วย เนื่องจาก เดิมทีมีเพียง ใส่ cp แล้วจบ
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">sku</t>
   </si>
@@ -50,6 +50,18 @@
   </si>
   <si>
     <t xml:space="preserve">CP2606160017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP2-001703+SP2-001596+SP2-001597+SP2-001598</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP2606160017 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">IP4-001747</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DC2606020003</t>
   </si>
 </sst>
 </file>
@@ -61,7 +73,7 @@
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Tahoma"/>
@@ -88,6 +100,17 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -98,7 +121,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -106,6 +129,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin">
+        <color rgb="FFF0F0F0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFF0F0F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -132,7 +166,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -141,6 +175,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -150,6 +188,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -162,6 +212,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFF0F0F0"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -276,15 +386,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultColWidth="11.74609375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="47.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="14.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="14.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="14.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.65"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.03"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -314,20 +426,57 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="4" t="n">
         <v>948</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="5" t="n">
         <v>46190</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="5" t="n">
         <v>46196</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>953</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>46190</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>46196</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>503</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>46175</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>46203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: process_price_mismatches() ปรับ logic
ปรับ logic การรับ input สำหรับการใช้ค่าของ oc dc ให้ทำงานตาม สถาปัตยกรรมของ fn overcharge_product และ discount_product เช่น หมึก 4 สี ลด 14, 10, 10, 10 บาท ตามลำดับ ก็ใส่ค่าเป็น 14 10 10 10
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/cp_data.xlsx
+++ b/projects/auto_page/autopageMKII/tables/cp_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t xml:space="preserve">sku</t>
   </si>
@@ -56,6 +56,9 @@
   </si>
   <si>
     <t xml:space="preserve">CP2606160017 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">12 10 10 10</t>
   </si>
   <si>
     <t xml:space="preserve">IP4-001747</t>
@@ -458,19 +461,19 @@
       <c r="E3" s="5" t="n">
         <v>46196</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>503</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>46175</v>

</xml_diff>